<commit_message>
Add first RAS findings batch
</commit_message>
<xml_diff>
--- a/content/ras-findings/batches/RAS-PR-batch1-doors-maneuvering-clearance.xlsx
+++ b/content/ras-findings/batches/RAS-PR-batch1-doors-maneuvering-clearance.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="105">
   <si>
     <t>RAS Plan Review Findings — Authoring Template (v1)</t>
   </si>
@@ -137,10 +137,10 @@
     <t>approved</t>
   </si>
   <si>
-    <t>Latch-side pull clearance</t>
-  </si>
-  <si>
-    <t>Plans show insufficient maneuvering clearance on the latch side at the pull side of the door. Provide dimensioned plan graphics confirming compliance with TAS 404.2.3.2 maneuvering clearance requirements.</t>
+    <t>Accessible maneuvering clearance not provided</t>
+  </si>
+  <si>
+    <t>Accessible maneuvering clearance is not provided on the pull side of the door [LOCATION] for a [forward | hinge | latch] approach.</t>
   </si>
   <si>
     <t>Doors</t>
@@ -167,7 +167,7 @@
     <t>10</t>
   </si>
   <si>
-    <t>Batch 1 seed — placeholder category/item</t>
+    <t>Placeholder category/item — not resolved</t>
   </si>
   <si>
     <t>true</t>
@@ -176,10 +176,10 @@
     <t>PR-B1-002</t>
   </si>
   <si>
-    <t>Hinge-side push clearance not shown</t>
-  </si>
-  <si>
-    <t>Insufficient information is provided to verify hinge-side maneuvering clearance on the push side of the door. Include enlarged door plans with required clearance dimensions.</t>
+    <t>Door maneuvering clearance cannot be determined</t>
+  </si>
+  <si>
+    <t>Insufficient information is provided to determine whether accessible maneuvering clearance is provided on the pull side of the door [LOCATION] for a [forward | hinge | latch] approach.</t>
   </si>
   <si>
     <t>insufficient_information</t>
@@ -191,121 +191,49 @@
     <t>PR-B1-003</t>
   </si>
   <si>
-    <t>Front-approach maneuvering clearance</t>
-  </si>
-  <si>
-    <t>Plans show the door approach does not provide the required front-approach maneuvering clearance. Clarify door location and dimensioned clearance on the architectural floor plans.</t>
-  </si>
-  <si>
-    <t>30</t>
+    <t>needs_review</t>
+  </si>
+  <si>
+    <t>Draft — pending reviewer approval</t>
   </si>
   <si>
     <t>PR-B1-004</t>
   </si>
   <si>
-    <t>Door swing conflicts with clearance</t>
-  </si>
-  <si>
-    <t>The drawings indicate the door swing conflicts with the required maneuvering clearance at the approach. Revise door handing or layout to coordinate swing with TAS 404.2.3 and 404.2.4.</t>
-  </si>
-  <si>
-    <t>404.2.3;404.2.4</t>
+    <t>skip</t>
+  </si>
+  <si>
+    <t>plan_review</t>
+  </si>
+  <si>
+    <t>Skip — duplicate of PR-B1-001</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Allowed value</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>tasRefs: semicolon-separated TAS 2012 refs or standard IDs (free text on Findings).</t>
+  </si>
+  <si>
+    <t>update</t>
+  </si>
+  <si>
+    <t>draft</t>
+  </si>
+  <si>
+    <t>rejected</t>
+  </si>
+  <si>
+    <t>imported</t>
   </si>
   <si>
     <t>coordination_issue</t>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>Compound — swing plus clearance</t>
-  </si>
-  <si>
-    <t>PR-B1-005</t>
-  </si>
-  <si>
-    <t>Recessed door maneuvering depth</t>
-  </si>
-  <si>
-    <t>Plans show a recessed door location without dimensioned maneuvering clearance depth at the recess. Provide plan details confirming compliance with TAS maneuvering clearance at recessed entries.</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>PR-B1-006</t>
-  </si>
-  <si>
-    <t>Maneuvering clearance not on plans</t>
-  </si>
-  <si>
-    <t>Insufficient information is provided to verify door maneuvering clearances on the submitted plans. Include dimensioned graphics for each required approach per TAS 404.2.3.</t>
-  </si>
-  <si>
-    <t>404.2.3</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>PR-B1-007</t>
-  </si>
-  <si>
-    <t>needs_review</t>
-  </si>
-  <si>
-    <t>Latch-side clearance draft</t>
-  </si>
-  <si>
-    <t>Plans show a restroom entry door; latch-side clearance graphics may be incomplete. Confirm wording and sheet references before approval.</t>
-  </si>
-  <si>
-    <t>plan_review;toilet_rooms</t>
-  </si>
-  <si>
-    <t>Draft — pending reviewer edit</t>
-  </si>
-  <si>
-    <t>PR-B1-008</t>
-  </si>
-  <si>
-    <t>skip</t>
-  </si>
-  <si>
-    <t>Duplicate maneuvering note</t>
-  </si>
-  <si>
-    <t>Plans show a door maneuvering clearance note that duplicates an existing library comment. Use existing row instead of importing a duplicate.</t>
-  </si>
-  <si>
-    <t>plan_review</t>
-  </si>
-  <si>
-    <t>Skip — duplicate of PR-B1-001 intent</t>
-  </si>
-  <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>Allowed value</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>tasRefs: semicolon-separated TAS 2012 refs or standard IDs (free text on Findings).</t>
-  </si>
-  <si>
-    <t>update</t>
-  </si>
-  <si>
-    <t>draft</t>
-  </si>
-  <si>
-    <t>rejected</t>
-  </si>
-  <si>
-    <t>imported</t>
   </si>
   <si>
     <t>best_practice</t>
@@ -899,7 +827,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1066,13 +994,13 @@
         <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F4" t="s">
         <v>41</v>
@@ -1087,7 +1015,7 @@
         <v>44</v>
       </c>
       <c r="J4" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="K4" t="s">
         <v>46</v>
@@ -1096,10 +1024,10 @@
         <v>47</v>
       </c>
       <c r="M4" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="N4" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="O4" t="s">
         <v>50</v>
@@ -1107,19 +1035,19 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" t="s">
         <v>60</v>
-      </c>
-      <c r="B5" t="s">
-        <v>37</v>
       </c>
       <c r="C5" t="s">
         <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="F5" t="s">
         <v>41</v>
@@ -1131,22 +1059,22 @@
         <v>43</v>
       </c>
       <c r="I5" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="J5" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="K5" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="L5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="M5" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="N5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="O5" t="s">
         <v>50</v>
@@ -1154,190 +1082,237 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="F6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
         <v>43</v>
       </c>
       <c r="I6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="L6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="M6" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="N6" t="s">
         <v>43</v>
       </c>
       <c r="O6" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H7" t="s">
         <v>43</v>
       </c>
       <c r="I7" t="s">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="J7" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="K7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="L7" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="M7" t="s">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="N7" t="s">
         <v>43</v>
       </c>
       <c r="O7" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>78</v>
+        <v>43</v>
       </c>
       <c r="E8" t="s">
-        <v>79</v>
+        <v>43</v>
       </c>
       <c r="F8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H8" t="s">
         <v>43</v>
       </c>
       <c r="I8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K8" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="L8" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="M8" t="s">
         <v>43</v>
       </c>
       <c r="N8" t="s">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="O8" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>82</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>84</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H9" t="s">
         <v>43</v>
       </c>
       <c r="I9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K9" t="s">
-        <v>86</v>
+        <v>43</v>
       </c>
       <c r="L9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="M9" t="s">
         <v>43</v>
       </c>
       <c r="N9" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="O9" t="s">
-        <v>50</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" t="s">
+        <v>43</v>
+      </c>
+      <c r="H10" t="s">
+        <v>43</v>
+      </c>
+      <c r="I10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J10" t="s">
+        <v>43</v>
+      </c>
+      <c r="K10" t="s">
+        <v>43</v>
+      </c>
+      <c r="L10" t="s">
+        <v>43</v>
+      </c>
+      <c r="M10" t="s">
+        <v>43</v>
+      </c>
+      <c r="N10" t="s">
+        <v>43</v>
+      </c>
+      <c r="O10" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1391,14 +1366,14 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2" t="s">
-        <v>90</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1409,17 +1384,17 @@
         <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>91</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>92</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1427,12 +1402,12 @@
         <v>23</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.25">
@@ -1442,12 +1417,12 @@
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>94</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -1465,22 +1440,22 @@
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -1511,50 +1486,50 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="D25" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>105</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1576,74 +1551,74 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>108</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>109</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="B5" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="B7" t="s">
-        <v>120</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>121</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
-        <v>122</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="B9" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1668,22 +1643,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>126</v>
+        <v>102</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>127</v>
+        <v>103</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>